<commit_message>
Stabilize capstone dashboard formatting
</commit_message>
<xml_diff>
--- a/tasks/Data Analytics Capstone Project/outputs/college_upload_files/02_google_sheets_dashboard.xlsx
+++ b/tasks/Data Analytics Capstone Project/outputs/college_upload_files/02_google_sheets_dashboard.xlsx
@@ -21,7 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
   <fonts count="13">
     <font>
       <name val="Calibri"/>
@@ -124,7 +127,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -146,11 +149,80 @@
         <color rgb="00D8DEE6"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D8DEE6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D8DEE6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D8DEE6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D8DEE6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D8DEE6"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D8DEE6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D8DEE6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D8DEE6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D8DEE6"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D8DEE6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -188,6 +260,30 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -288,6 +384,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -313,6 +412,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -338,6 +440,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -363,6 +468,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -393,6 +501,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -418,6 +529,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -739,35 +853,35 @@
           <t>Workplace Mental Health Disclosure And Support Dashboard</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="2" t="n"/>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="16" t="n"/>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="16" t="n"/>
+      <c r="H1" s="16" t="n"/>
+      <c r="I1" s="16" t="n"/>
+      <c r="J1" s="16" t="n"/>
+      <c r="K1" s="16" t="n"/>
+      <c r="L1" s="16" t="n"/>
+      <c r="M1" s="16" t="n"/>
+      <c r="N1" s="17" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
+      <c r="A2" s="18" t="n"/>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="19" t="n"/>
+      <c r="E2" s="19" t="n"/>
+      <c r="F2" s="19" t="n"/>
+      <c r="G2" s="19" t="n"/>
+      <c r="H2" s="19" t="n"/>
+      <c r="I2" s="19" t="n"/>
+      <c r="J2" s="19" t="n"/>
+      <c r="K2" s="19" t="n"/>
+      <c r="L2" s="19" t="n"/>
+      <c r="M2" s="19" t="n"/>
+      <c r="N2" s="20" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -775,35 +889,35 @@
           <t>OSMI Mental Health in Tech Survey | Main story: treatment-seeking is common, but workplace disclosure comfort remains much lower.</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="16" t="n"/>
+      <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
+      <c r="J3" s="16" t="n"/>
+      <c r="K3" s="16" t="n"/>
+      <c r="L3" s="16" t="n"/>
+      <c r="M3" s="16" t="n"/>
+      <c r="N3" s="17" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
+      <c r="A4" s="18" t="n"/>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+      <c r="F4" s="19" t="n"/>
+      <c r="G4" s="19" t="n"/>
+      <c r="H4" s="19" t="n"/>
+      <c r="I4" s="19" t="n"/>
+      <c r="J4" s="19" t="n"/>
+      <c r="K4" s="19" t="n"/>
+      <c r="L4" s="19" t="n"/>
+      <c r="M4" s="19" t="n"/>
+      <c r="N4" s="20" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1">
@@ -813,60 +927,56 @@
 1259</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
+      <c r="B6" s="16" t="n"/>
+      <c r="C6" s="17" t="n"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Sought treatment
 637 respondents (50.6%)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="17" t="n"/>
       <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Know benefits
 477 respondents (37.9%)</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="17" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
           <t>Any work interference
 782 respondents (62.1%)</t>
         </is>
       </c>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
+      <c r="K6" s="16" t="n"/>
+      <c r="L6" s="17" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
+      <c r="A7" s="21" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="21" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="21" t="n"/>
+      <c r="L7" s="22" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
+      <c r="A8" s="18" t="n"/>
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="20" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="20" t="n"/>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="19" t="n"/>
+      <c r="I8" s="20" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="19" t="n"/>
+      <c r="L8" s="20" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1"/>
     <row r="10" ht="24" customHeight="1">
@@ -876,60 +986,52 @@
 516 respondents (41.0%)</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
+      <c r="B10" s="16" t="n"/>
+      <c r="C10" s="17" t="n"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Coworker comfort
 225 respondents (17.9%)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="17" t="n"/>
       <c r="G10" s="8" t="inlineStr">
         <is>
           <t>Interpretation: benefit/care-option awareness, work interference, and perceived consequences are strongly associated with treatment-seeking or disclosure comfort. Results are associations, not causal claims.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
+      <c r="H10" s="16" t="n"/>
+      <c r="I10" s="16" t="n"/>
+      <c r="J10" s="16" t="n"/>
+      <c r="K10" s="16" t="n"/>
+      <c r="L10" s="16" t="n"/>
+      <c r="M10" s="16" t="n"/>
+      <c r="N10" s="17" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
+      <c r="A11" s="21" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="F11" s="22" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="N11" s="22" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
+      <c r="A12" s="18" t="n"/>
+      <c r="B12" s="19" t="n"/>
+      <c r="C12" s="20" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="20" t="n"/>
+      <c r="G12" s="18" t="n"/>
+      <c r="H12" s="19" t="n"/>
+      <c r="I12" s="19" t="n"/>
+      <c r="J12" s="19" t="n"/>
+      <c r="K12" s="19" t="n"/>
+      <c r="L12" s="19" t="n"/>
+      <c r="M12" s="19" t="n"/>
+      <c r="N12" s="20" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1"/>
     <row r="14" ht="24" customHeight="1"/>
@@ -971,51 +1073,39 @@
           <t>Dashboard source: OSMI Mental Health in Tech Survey via Kaggle. Use Additional_Charts, Source_Tables, Hypothesis_Tests, and Model sheets for audit details.</t>
         </is>
       </c>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n"/>
-      <c r="J47" s="2" t="n"/>
-      <c r="K47" s="2" t="n"/>
-      <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="n"/>
-      <c r="N47" s="2" t="n"/>
+      <c r="B47" s="16" t="n"/>
+      <c r="C47" s="16" t="n"/>
+      <c r="D47" s="16" t="n"/>
+      <c r="E47" s="16" t="n"/>
+      <c r="F47" s="16" t="n"/>
+      <c r="G47" s="16" t="n"/>
+      <c r="H47" s="16" t="n"/>
+      <c r="I47" s="16" t="n"/>
+      <c r="J47" s="16" t="n"/>
+      <c r="K47" s="16" t="n"/>
+      <c r="L47" s="16" t="n"/>
+      <c r="M47" s="16" t="n"/>
+      <c r="N47" s="17" t="n"/>
     </row>
     <row r="48" ht="24" customHeight="1">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
-      <c r="J48" s="2" t="n"/>
-      <c r="K48" s="2" t="n"/>
-      <c r="L48" s="2" t="n"/>
-      <c r="M48" s="2" t="n"/>
-      <c r="N48" s="2" t="n"/>
+      <c r="A48" s="21" t="n"/>
+      <c r="N48" s="22" t="n"/>
     </row>
     <row r="49" ht="24" customHeight="1">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
-      <c r="G49" s="2" t="n"/>
-      <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="n"/>
-      <c r="J49" s="2" t="n"/>
-      <c r="K49" s="2" t="n"/>
-      <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="n"/>
-      <c r="N49" s="2" t="n"/>
+      <c r="A49" s="18" t="n"/>
+      <c r="B49" s="19" t="n"/>
+      <c r="C49" s="19" t="n"/>
+      <c r="D49" s="19" t="n"/>
+      <c r="E49" s="19" t="n"/>
+      <c r="F49" s="19" t="n"/>
+      <c r="G49" s="19" t="n"/>
+      <c r="H49" s="19" t="n"/>
+      <c r="I49" s="19" t="n"/>
+      <c r="J49" s="19" t="n"/>
+      <c r="K49" s="19" t="n"/>
+      <c r="L49" s="19" t="n"/>
+      <c r="M49" s="19" t="n"/>
+      <c r="N49" s="20" t="n"/>
     </row>
     <row r="50" ht="24" customHeight="1"/>
     <row r="51" ht="24" customHeight="1"/>
@@ -1217,7 +1307,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Dashboard Source Tables</t>
         </is>
@@ -1225,14 +1315,14 @@
     </row>
     <row r="2" ht="24" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>Treatment by benefits</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>benefits</t>
         </is>
@@ -1259,7 +1349,7 @@
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1278,7 +1368,7 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1297,7 +1387,7 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Don't know</t>
         </is>
@@ -1318,14 +1408,14 @@
     <row r="8" ht="24" customHeight="1"/>
     <row r="9" ht="24" customHeight="1"/>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Treatment by care options</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>care_options</t>
         </is>
@@ -1352,7 +1442,7 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1371,7 +1461,7 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1390,7 +1480,7 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Not sure</t>
         </is>
@@ -1411,14 +1501,14 @@
     <row r="15" ht="24" customHeight="1"/>
     <row r="16" ht="24" customHeight="1"/>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>Treatment by work interference</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>work_interfere</t>
         </is>
@@ -1445,7 +1535,7 @@
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Often</t>
         </is>
@@ -1464,7 +1554,7 @@
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>Sometimes</t>
         </is>
@@ -1483,7 +1573,7 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Rarely</t>
         </is>
@@ -1502,7 +1592,7 @@
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Never</t>
         </is>
@@ -1521,7 +1611,7 @@
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
@@ -1542,14 +1632,14 @@
     <row r="24" ht="24" customHeight="1"/>
     <row r="25" ht="24" customHeight="1"/>
     <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="A26" s="24" t="inlineStr">
         <is>
           <t>Treatment by company size</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="25" t="inlineStr">
         <is>
           <t>company_size</t>
         </is>
@@ -1576,130 +1666,130 @@
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>1 to 5</t>
         </is>
       </c>
-      <c r="B28" s="14" t="n">
+      <c r="B28" s="27" t="n">
         <v>162</v>
       </c>
-      <c r="C28" s="14" t="n">
+      <c r="C28" s="27" t="n">
         <v>91</v>
       </c>
-      <c r="D28" s="14" t="n">
+      <c r="D28" s="28" t="n">
         <v>0.5617283950617284</v>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="29" t="n">
         <v>56.2</v>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>6 to 25</t>
         </is>
       </c>
-      <c r="B29" s="14" t="n">
+      <c r="B29" s="27" t="n">
         <v>290</v>
       </c>
-      <c r="C29" s="14" t="n">
+      <c r="C29" s="27" t="n">
         <v>128</v>
       </c>
-      <c r="D29" s="14" t="n">
+      <c r="D29" s="28" t="n">
         <v>0.4413793103448276</v>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="E29" s="29" t="n">
         <v>44.1</v>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" s="26" t="inlineStr">
         <is>
           <t>26 to 100</t>
         </is>
       </c>
-      <c r="B30" s="14" t="n">
+      <c r="B30" s="27" t="n">
         <v>289</v>
       </c>
-      <c r="C30" s="14" t="n">
+      <c r="C30" s="27" t="n">
         <v>150</v>
       </c>
-      <c r="D30" s="14" t="n">
+      <c r="D30" s="28" t="n">
         <v>0.5190311418685121</v>
       </c>
-      <c r="E30" s="14" t="n">
+      <c r="E30" s="29" t="n">
         <v>51.9</v>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="26" t="inlineStr">
         <is>
           <t>100 to 500</t>
         </is>
       </c>
-      <c r="B31" s="14" t="n">
+      <c r="B31" s="27" t="n">
         <v>176</v>
       </c>
-      <c r="C31" s="14" t="n">
+      <c r="C31" s="27" t="n">
         <v>95</v>
       </c>
-      <c r="D31" s="14" t="n">
+      <c r="D31" s="28" t="n">
         <v>0.5397727272727273</v>
       </c>
-      <c r="E31" s="14" t="n">
+      <c r="E31" s="29" t="n">
         <v>54</v>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="A32" s="26" t="inlineStr">
         <is>
           <t>500 to 1000</t>
         </is>
       </c>
-      <c r="B32" s="14" t="n">
+      <c r="B32" s="27" t="n">
         <v>60</v>
       </c>
-      <c r="C32" s="14" t="n">
+      <c r="C32" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="D32" s="14" t="n">
+      <c r="D32" s="28" t="n">
         <v>0.45</v>
       </c>
-      <c r="E32" s="14" t="n">
+      <c r="E32" s="29" t="n">
         <v>45</v>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="14" t="inlineStr">
+      <c r="A33" s="26" t="inlineStr">
         <is>
           <t>More than 1000</t>
         </is>
       </c>
-      <c r="B33" s="14" t="n">
+      <c r="B33" s="27" t="n">
         <v>282</v>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C33" s="27" t="n">
         <v>146</v>
       </c>
-      <c r="D33" s="14" t="n">
+      <c r="D33" s="28" t="n">
         <v>0.5177304964539007</v>
       </c>
-      <c r="E33" s="14" t="n">
+      <c r="E33" s="29" t="n">
         <v>51.8</v>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1"/>
     <row r="35" ht="24" customHeight="1"/>
     <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="A36" s="24" t="inlineStr">
         <is>
           <t>Treatment by family history</t>
         </is>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>family_history</t>
         </is>
@@ -1726,7 +1816,7 @@
       </c>
     </row>
     <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="A38" s="26" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1745,7 +1835,7 @@
       </c>
     </row>
     <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="A39" s="26" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>